<commit_message>
labeling for all original_correct sample and feature adapted by logit
</commit_message>
<xml_diff>
--- a/experiment/實驗結果.xlsx
+++ b/experiment/實驗結果.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ted\Desktop\論文\experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC669D19-5121-4B68-B23A-09ACFA85D764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D00E03FF-9BC9-4D0D-BF7E-0CAE5792AEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3ECA1DB8-1BD9-46FA-B4F1-485F2799EAA5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="70">
   <si>
     <t>調整label設定後</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -141,14 +141,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>直接用feature差異訓練fuzzy detector</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>用feature的shap簽名差異訓練fuzzy detector</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>0.7567</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -198,6 +190,134 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>用feature(128)的shap簽名差異訓練fuzzy detector</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>用feature(logit)的shap簽名差異訓練fuzzy detector</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9633</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9700</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9569</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>51</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.6290</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>626/1000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>eps=0.352</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9467</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9333</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9422</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>43</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.4360</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>435/1000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>eps=0.222,iter=103</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>直接用feature(128)差異訓練fuzzy detector</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>直接用feature(logit)差異訓練fuzzy detector</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.8533</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9095</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.7551</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.7810</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>781/1000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.8100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.8421</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.8032</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.6230</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>623/1000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">eps=0.437 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">eps=0.253,iter=146 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>61</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>63</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -597,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11F37ECD-1310-4DB8-985C-13F95F33B97D}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.75" style="1" bestFit="1" customWidth="1"/>
@@ -617,7 +737,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -700,7 +820,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -734,25 +854,25 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -760,30 +880,196 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="1" t="s">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I17" s="1" t="s">
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feature fuzzy detector+shap fuzzy detector v2
</commit_message>
<xml_diff>
--- a/experiment/實驗結果.xlsx
+++ b/experiment/實驗結果.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ted\Desktop\論文\experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D00E03FF-9BC9-4D0D-BF7E-0CAE5792AEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9B06C5-D6F9-47FC-B348-1F4A9FE1BA37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3ECA1DB8-1BD9-46FA-B4F1-485F2799EAA5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="60">
   <si>
     <t>調整label設定後</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -61,10 +61,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve"> Successful/Total</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Params</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -109,10 +105,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>365/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">eps=0.272 </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -133,10 +125,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>473/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">eps=0.234,iter=91 </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -157,10 +145,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>686/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>eps=0.401</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -181,10 +165,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>426/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>eps=0.224,iter=105</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -201,62 +181,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>0.9633</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.9700</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.9569</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>51</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.6290</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>626/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>eps=0.352</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.9467</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.9333</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.9422</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>43</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.4360</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>435/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>eps=0.222,iter=103</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>直接用feature(128)差異訓練fuzzy detector</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -265,59 +189,94 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>0.8533</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.9095</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.7551</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.7810</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>781/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.8100</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.8421</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.8032</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0.6230</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>623/1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">eps=0.437 </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">eps=0.253,iter=146 </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>61</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>63</t>
+    <t>0.9850</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9860</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9799</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>33</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.4840</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>eps=0.297</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9883</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9879</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9846</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.3900</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">eps=0.214,iter=91 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.7117</t>
+  </si>
+  <si>
+    <t>0.7343</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.7090</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>57</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.6660</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.9260</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>56</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.6378</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.6635</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.6450</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">eps=0.371 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>eps=0.364,iter=130</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -717,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11F37ECD-1310-4DB8-985C-13F95F33B97D}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.75" style="1" bestFit="1" customWidth="1"/>
@@ -726,26 +685,26 @@
     <col min="4" max="4" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="17.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="7" max="7" width="17.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>1</v>
@@ -762,73 +721,64 @@
       <c r="G4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>1</v>
@@ -845,73 +795,64 @@
       <c r="G9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>1</v>
@@ -928,78 +869,69 @@
       <c r="G14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="2" t="s">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H17" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I17" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>1</v>
@@ -1016,60 +948,51 @@
       <c r="G19" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="H20" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>